<commit_message>
feat: Luban 切分 dev/release 管线，开发期用 JSON 数据源
</commit_message>
<xml_diff>
--- a/Config/Datas/PipelineData.xlsx
+++ b/Config/Datas/PipelineData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>##var</t>
   </si>
@@ -56,22 +56,10 @@
     <t>名称</t>
   </si>
   <si>
-    <t>通用-出生</t>
-  </si>
-  <si>
-    <t>雅-普通攻击-1</t>
-  </si>
-  <si>
-    <t>雅-普通攻击-2</t>
-  </si>
-  <si>
-    <t>雅-普通攻击-3</t>
-  </si>
-  <si>
-    <t>雅-普通攻击-4</t>
-  </si>
-  <si>
-    <t>雅-死亡进行-1</t>
+    <t>出生进行</t>
+  </si>
+  <si>
+    <t>死亡进行</t>
   </si>
   <si>
     <t>剑-翻滚</t>
@@ -1105,8 +1093,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4" outlineLevelCol="2"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4" outlineLevelRow="6" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="3" width="21.712962962963" style="2" customWidth="1"/>
@@ -1163,7 +1151,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="B6" s="2">
-        <v>10002</v>
+        <v>10020</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -1171,42 +1159,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="B7" s="2">
-        <v>10003</v>
+        <v>10030</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="B8" s="2">
-        <v>10004</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="B9" s="2">
-        <v>10010</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="B10" s="2">
-        <v>10020</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="B11" s="2">
-        <v>10030</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>